<commit_message>
LSA Design System: fix Experience Workspace (md2jcr) mapping
- lsa-* block definitions: title and template name "Lsa Hero", "Lsa Give Band",
  "Lsa News", "Lsa Swatches" (md2jcr matches the document's block name, which the
  pipeline title-cases, against the definition title exactly). "LSA Hero" failed
  with "The component 'Lsa Hero' does not exist".
- columns: the LSA DS image + text variant is now the single-word `media`
  (scoped to body.lsa-ds); md2jcr turned "lsa-media" into classes "lsa media".
  Columns model gets a Style (classes) select so the variant is kept and editable.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-figma.report.xlsx
+++ b/tools/importer/reports/import-figma.report.xlsx
@@ -286,7 +286,7 @@
     <t>en/lsa-figma/index</t>
   </si>
   <si>
-    <t>2026-10-26T18:36:57.655Z</t>
+    <t>2026-10-26T19:37:40.260Z</t>
   </si>
   <si>
     <t>LSA Design System</t>
@@ -316,7 +316,7 @@
     <t>en/lsa-figma/style-guide</t>
   </si>
   <si>
-    <t>2026-10-26T18:37:04.346Z</t>
+    <t>2026-10-26T19:37:44.774Z</t>
   </si>
   <si>
     <t>LSA Design System – Style Guide</t>

</xml_diff>

<commit_message>
Why LSA page source (/en/lsa-figma/why-lsa)
From the Figma "Why LSA" file (RpnIZdSskdoUmQiEcxY5Tt). The Figma API was
rate-limited, so the page is built from the exported hero image only
(media-da/lsa-figma/why-lsa-hero.png in DA): LSA Page Title (breadcrumb +
"Why LSA") and LSA Hero (photo), theme lsa-ds with the lsa-figma nav/footer.
Added to urls-figma.txt so build-da-docs includes it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-figma.report.xlsx
+++ b/tools/importer/reports/import-figma.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="309">
   <si>
     <t>_reportFile</t>
   </si>
@@ -368,6 +368,21 @@
   </si>
   <si>
     <t>http://localhost:8093/lsa-figma/style-guide.html</t>
+  </si>
+  <si>
+    <t>en/lsa-figma/why-lsa.report.json</t>
+  </si>
+  <si>
+    <t>en/lsa-figma/why-lsa</t>
+  </si>
+  <si>
+    <t>2026-10-28T16:28:25.878Z</t>
+  </si>
+  <si>
+    <t>Why LSA</t>
+  </si>
+  <si>
+    <t>http://localhost:8093/lsa-figma/why-lsa.html</t>
   </si>
   <si>
     <t>en/prospective-students/graduate.report.json</t>
@@ -1311,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -2000,7 +2015,7 @@
         <v>119</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -2008,46 +2023,46 @@
       <c r="D22" t="s">
         <v>120</v>
       </c>
-      <c r="E22" t="s">
-        <v>12</v>
+      <c r="E22">
+        <v>2</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="G22" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" t="s">
         <v>121</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>122</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>123</v>
-      </c>
-      <c r="J22" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
         <v>125</v>
       </c>
-      <c r="B23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
         <v>126</v>
-      </c>
-      <c r="E23" t="s">
-        <v>12</v>
-      </c>
-      <c r="F23" t="s">
-        <v>14</v>
-      </c>
-      <c r="G23" t="s">
-        <v>121</v>
       </c>
       <c r="H23" t="s">
         <v>127</v>
@@ -2079,7 +2094,7 @@
         <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H24" t="s">
         <v>132</v>
@@ -2096,7 +2111,7 @@
         <v>135</v>
       </c>
       <c r="B25" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
@@ -2111,7 +2126,7 @@
         <v>14</v>
       </c>
       <c r="G25" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H25" t="s">
         <v>137</v>
@@ -2128,7 +2143,7 @@
         <v>140</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -2143,7 +2158,7 @@
         <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H26" t="s">
         <v>142</v>
@@ -2160,39 +2175,39 @@
         <v>145</v>
       </c>
       <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
         <v>146</v>
       </c>
-      <c r="C27" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>126</v>
+      </c>
+      <c r="H27" t="s">
         <v>147</v>
       </c>
-      <c r="E27" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" t="s">
-        <v>14</v>
-      </c>
-      <c r="G27" t="s">
-        <v>50</v>
-      </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>148</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>149</v>
-      </c>
-      <c r="J27" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>150</v>
+      </c>
+      <c r="B28" t="s">
         <v>151</v>
-      </c>
-      <c r="B28" t="s">
-        <v>20</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -2207,7 +2222,7 @@
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>121</v>
+        <v>50</v>
       </c>
       <c r="H28" t="s">
         <v>153</v>
@@ -2239,7 +2254,7 @@
         <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>22</v>
+        <v>126</v>
       </c>
       <c r="H29" t="s">
         <v>158</v>
@@ -2256,7 +2271,7 @@
         <v>161</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -2277,24 +2292,24 @@
         <v>163</v>
       </c>
       <c r="I30" t="s">
-        <v>82</v>
+        <v>164</v>
       </c>
       <c r="J30" t="s">
-        <v>83</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B31" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="C31" t="s">
         <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E31" t="s">
         <v>12</v>
@@ -2306,45 +2321,45 @@
         <v>22</v>
       </c>
       <c r="H31" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I31" t="s">
-        <v>159</v>
+        <v>82</v>
       </c>
       <c r="J31" t="s">
-        <v>160</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>168</v>
-      </c>
-      <c r="E32">
-        <v>1</v>
+        <v>170</v>
+      </c>
+      <c r="E32" t="s">
+        <v>12</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="H32" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="I32" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="J32" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -2352,39 +2367,39 @@
         <v>172</v>
       </c>
       <c r="B33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" t="s">
         <v>173</v>
       </c>
-      <c r="C33" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>28</v>
+      </c>
+      <c r="H33" t="s">
         <v>174</v>
       </c>
-      <c r="E33" t="s">
-        <v>12</v>
-      </c>
-      <c r="F33" t="s">
-        <v>14</v>
-      </c>
-      <c r="G33" t="s">
-        <v>121</v>
-      </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>175</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>176</v>
-      </c>
-      <c r="J33" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>177</v>
+      </c>
+      <c r="B34" t="s">
         <v>178</v>
-      </c>
-      <c r="B34" t="s">
-        <v>173</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -2399,7 +2414,7 @@
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H34" t="s">
         <v>180</v>
@@ -2416,7 +2431,7 @@
         <v>183</v>
       </c>
       <c r="B35" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C35" t="s">
         <v>12</v>
@@ -2431,7 +2446,7 @@
         <v>14</v>
       </c>
       <c r="G35" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H35" t="s">
         <v>185</v>
@@ -2448,7 +2463,7 @@
         <v>188</v>
       </c>
       <c r="B36" t="s">
-        <v>20</v>
+        <v>178</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2463,7 +2478,7 @@
         <v>14</v>
       </c>
       <c r="G36" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H36" t="s">
         <v>190</v>
@@ -2495,7 +2510,7 @@
         <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H37" t="s">
         <v>195</v>
@@ -2527,7 +2542,7 @@
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H38" t="s">
         <v>200</v>
@@ -2559,7 +2574,7 @@
         <v>14</v>
       </c>
       <c r="G39" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H39" t="s">
         <v>205</v>
@@ -2591,7 +2606,7 @@
         <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H40" t="s">
         <v>210</v>
@@ -2623,7 +2638,7 @@
         <v>14</v>
       </c>
       <c r="G41" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H41" t="s">
         <v>215</v>
@@ -2655,7 +2670,7 @@
         <v>14</v>
       </c>
       <c r="G42" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H42" t="s">
         <v>220</v>
@@ -2687,7 +2702,7 @@
         <v>14</v>
       </c>
       <c r="G43" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H43" t="s">
         <v>225</v>
@@ -2719,7 +2734,7 @@
         <v>14</v>
       </c>
       <c r="G44" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H44" t="s">
         <v>230</v>
@@ -2751,7 +2766,7 @@
         <v>14</v>
       </c>
       <c r="G45" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H45" t="s">
         <v>235</v>
@@ -2783,7 +2798,7 @@
         <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H46" t="s">
         <v>240</v>
@@ -2815,7 +2830,7 @@
         <v>14</v>
       </c>
       <c r="G47" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H47" t="s">
         <v>245</v>
@@ -2847,7 +2862,7 @@
         <v>14</v>
       </c>
       <c r="G48" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H48" t="s">
         <v>250</v>
@@ -2879,30 +2894,30 @@
         <v>14</v>
       </c>
       <c r="G49" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H49" t="s">
         <v>255</v>
       </c>
       <c r="I49" t="s">
-        <v>201</v>
+        <v>256</v>
       </c>
       <c r="J49" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="C50" t="s">
         <v>12</v>
       </c>
       <c r="D50" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E50" t="s">
         <v>12</v>
@@ -2911,13 +2926,13 @@
         <v>14</v>
       </c>
       <c r="G50" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H50" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="I50" t="s">
-        <v>260</v>
+        <v>206</v>
       </c>
       <c r="J50" t="s">
         <v>261</v>
@@ -2928,7 +2943,7 @@
         <v>262</v>
       </c>
       <c r="B51" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="C51" t="s">
         <v>12</v>
@@ -2943,7 +2958,7 @@
         <v>14</v>
       </c>
       <c r="G51" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H51" t="s">
         <v>264</v>
@@ -2975,7 +2990,7 @@
         <v>14</v>
       </c>
       <c r="G52" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H52" t="s">
         <v>269</v>
@@ -2992,7 +3007,7 @@
         <v>272</v>
       </c>
       <c r="B53" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="C53" t="s">
         <v>12</v>
@@ -3007,7 +3022,7 @@
         <v>14</v>
       </c>
       <c r="G53" t="s">
-        <v>22</v>
+        <v>126</v>
       </c>
       <c r="H53" t="s">
         <v>274</v>
@@ -3045,42 +3060,42 @@
         <v>279</v>
       </c>
       <c r="I54" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="J54" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>282</v>
+      </c>
+      <c r="B55" t="s">
+        <v>79</v>
+      </c>
+      <c r="C55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" t="s">
+        <v>283</v>
+      </c>
+      <c r="E55" t="s">
+        <v>12</v>
+      </c>
+      <c r="F55" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" t="s">
+        <v>22</v>
+      </c>
+      <c r="H55" t="s">
+        <v>284</v>
+      </c>
+      <c r="I55" t="s">
         <v>280</v>
       </c>
-      <c r="B55" t="s">
-        <v>20</v>
-      </c>
-      <c r="C55" t="s">
-        <v>12</v>
-      </c>
-      <c r="D55" t="s">
+      <c r="J55" t="s">
         <v>281</v>
-      </c>
-      <c r="E55" t="s">
-        <v>12</v>
-      </c>
-      <c r="F55" t="s">
-        <v>14</v>
-      </c>
-      <c r="G55" t="s">
-        <v>121</v>
-      </c>
-      <c r="H55" t="s">
-        <v>282</v>
-      </c>
-      <c r="I55" t="s">
-        <v>283</v>
-      </c>
-      <c r="J55" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
@@ -3088,7 +3103,7 @@
         <v>285</v>
       </c>
       <c r="B56" t="s">
-        <v>173</v>
+        <v>20</v>
       </c>
       <c r="C56" t="s">
         <v>12</v>
@@ -3103,7 +3118,7 @@
         <v>14</v>
       </c>
       <c r="G56" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H56" t="s">
         <v>287</v>
@@ -3120,7 +3135,7 @@
         <v>290</v>
       </c>
       <c r="B57" t="s">
-        <v>20</v>
+        <v>178</v>
       </c>
       <c r="C57" t="s">
         <v>12</v>
@@ -3135,7 +3150,7 @@
         <v>14</v>
       </c>
       <c r="G57" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H57" t="s">
         <v>292</v>
@@ -3167,21 +3182,21 @@
         <v>14</v>
       </c>
       <c r="G58" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H58" t="s">
         <v>297</v>
       </c>
       <c r="I58" t="s">
-        <v>265</v>
+        <v>298</v>
       </c>
       <c r="J58" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B59" t="s">
         <v>20</v>
@@ -3190,7 +3205,7 @@
         <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E59" t="s">
         <v>12</v>
@@ -3199,16 +3214,48 @@
         <v>14</v>
       </c>
       <c r="G59" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H59" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I59" t="s">
-        <v>302</v>
+        <v>270</v>
       </c>
       <c r="J59" t="s">
         <v>303</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>304</v>
+      </c>
+      <c r="B60" t="s">
+        <v>20</v>
+      </c>
+      <c r="C60" t="s">
+        <v>12</v>
+      </c>
+      <c r="D60" t="s">
+        <v>305</v>
+      </c>
+      <c r="E60" t="s">
+        <v>12</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60" t="s">
+        <v>126</v>
+      </c>
+      <c r="H60" t="s">
+        <v>306</v>
+      </c>
+      <c r="I60" t="s">
+        <v>307</v>
+      </c>
+      <c r="J60" t="s">
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>